<commit_message>
Implement academic hierarchy (School/Dept -> Degree -> Batch -> Semester -> Subject) for creation, bulk uploads, and cascading generation dropdowns
</commit_message>
<xml_diff>
--- a/public/subjects-template.xlsx
+++ b/public/subjects-template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Subjects" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Faculty" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -72,15 +72,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,26 +449,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="45" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Degree Program</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Batch</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Semester</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Subject Code</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Subject Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>CO Count</t>
         </is>
@@ -474,61 +501,186 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>SOES</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>B.Tech CSE</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2023-2027</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>CAP1005</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Programming and Problem Solving Using C</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>5</v>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Data Structures and Algorithms</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>CAP1006</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Object Oriented Programming using Java</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>5</v>
+          <t>SOES</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>BCA</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2024-2027</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>CAP1001</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Problem Solving Using C</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>CAP1007</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Database Management Systems</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>5</v>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>BA LLB</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2022-2027</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>LAW2003</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Constitutional Law II</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>CAP2001</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Data Structures and Algorithms</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>6</v>
+          <t>SOHAS</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>B.Sc Physics</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2024-2027</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>PHY1001</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Classical Mechanics</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SOB</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>BBA</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>2023-2026</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>MGT2001</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Financial Management</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restrict batch year to single 4-digit calendar year (e.g. 2023) across creation form, templates, and parsers
</commit_message>
<xml_diff>
--- a/public/subjects-template.xlsx
+++ b/public/subjects-template.xlsx
@@ -474,7 +474,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Batch</t>
+          <t>Batch Year</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -511,7 +511,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2023-2027</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -548,7 +548,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2024-2027</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -585,7 +585,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2022-2027</t>
+          <t>2022</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2024-2027</t>
+          <t>2024</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -659,7 +659,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2023-2026</t>
+          <t>2023</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">

</xml_diff>